<commit_message>
test(newman): mở rộng độ phủ thực thi lên >=90% và thêm báo cáo đối soát
</commit_message>
<xml_diff>
--- a/hw06/excel/test-cases.xlsx
+++ b/hw06/excel/test-cases.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HW06 test cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'HW06 test cases'!$A$1:$K$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'HW06 test cases'!$A$1:$M$129</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K129"/>
+  <dimension ref="A1:M129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,8 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,6 +499,16 @@
           <t>Bug ID</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Lý do</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -554,6 +566,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -611,6 +633,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -668,6 +700,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -725,6 +767,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -782,6 +834,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -839,6 +901,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -896,6 +968,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -953,6 +1035,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1010,6 +1102,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1067,6 +1169,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1124,6 +1236,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1181,6 +1303,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1238,6 +1370,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1295,6 +1437,16 @@
           <t>D-LOGIN-08</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1352,6 +1504,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1409,6 +1571,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1466,6 +1638,16 @@
           <t>D-LOGIN-01</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1523,6 +1705,16 @@
           <t>D-LOGIN-01</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1580,6 +1772,16 @@
           <t>D-LOGIN-01</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1637,6 +1839,16 @@
           <t>D-LOGIN-07</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1694,6 +1906,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1751,6 +1973,16 @@
           <t>D-LOGIN-02</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1808,6 +2040,16 @@
           <t>D-LOGIN-01</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1865,6 +2107,16 @@
           <t>D-LOGIN-01</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Tiền điều kiện yêu cầu TC-023 đăng nhập thành công sau hai lần sai, nhưng D-LOGIN-01 khóa tài khoản sớm nên không thể đi tới trạng thái reset cần kiểm thử.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1922,6 +2174,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1979,6 +2241,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2036,6 +2308,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2093,6 +2375,16 @@
           <t>D-LOGIN-03</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2150,6 +2442,16 @@
           <t>D-LOGIN-03</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2207,6 +2509,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2264,6 +2576,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2321,6 +2643,16 @@
           <t>D-LOGIN-07</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2378,6 +2710,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2435,6 +2777,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2492,6 +2844,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2549,6 +2911,16 @@
           <t>D-LOGIN-03</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2606,6 +2978,16 @@
           <t>D-LOGIN-01</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2663,6 +3045,16 @@
           <t>D-LOGIN-02</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2720,6 +3112,16 @@
           <t>D-LOGIN-03</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2777,6 +3179,16 @@
           <t>D-LOGIN-05</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2834,6 +3246,16 @@
           <t>D-LOGIN-06</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Phải chờ lock thực tế 180 giây rồi kiểm tra residual state; tách khỏi regression tự động để tránh một iteration kéo dài và dễ nhiễu thời gian.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2891,6 +3313,16 @@
           <t>D-LOGIN-05</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Cần ký JWT bằng secret của SUT; không nhúng signing secret hoặc forged token vào collection/report công khai.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2948,6 +3380,16 @@
           <t>D-CHK-01</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3005,6 +3447,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3062,6 +3514,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3119,6 +3581,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3176,6 +3648,16 @@
           <t>D-CHK-02</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3233,6 +3715,16 @@
           <t>D-CHK-02</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3290,6 +3782,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3347,6 +3849,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3404,6 +3916,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3461,6 +3983,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3518,6 +4050,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3575,6 +4117,16 @@
           <t>D-CHK-05</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3632,6 +4184,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3689,6 +4251,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3746,6 +4318,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3803,6 +4385,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3860,6 +4452,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3917,6 +4519,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3974,6 +4586,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4031,6 +4653,16 @@
           <t>D-CHK-03</t>
         </is>
       </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4088,6 +4720,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4145,6 +4787,16 @@
           <t>D-CHK-04</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4202,6 +4854,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4259,6 +4921,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4316,6 +4988,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4373,6 +5055,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4430,6 +5122,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4487,6 +5189,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4544,6 +5256,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>SUT phát JWT không có exp và không cung cấp signing fixture an toàn, nên không thể tạo token hợp lệ nhưng đã hết hạn mà không sao chép secret vào artifact.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4601,6 +5323,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4658,6 +5390,16 @@
           <t>D-CHK-07</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4715,6 +5457,16 @@
           <t>D-CHK-05</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4772,6 +5524,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4829,6 +5591,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4886,6 +5658,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4943,6 +5725,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5000,6 +5792,16 @@
           <t>D-CHK-01</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5057,6 +5859,16 @@
           <t>D-CHK-02</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5114,6 +5926,16 @@
           <t>D-CHK-03</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5171,6 +5993,16 @@
           <t>D-CHK-04</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5228,6 +6060,16 @@
           <t>D-CHK-07</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5285,6 +6127,16 @@
           <t>D-CHK-05</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5342,6 +6194,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5399,6 +6261,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5456,6 +6328,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5513,6 +6395,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5570,6 +6462,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5627,6 +6529,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5684,6 +6596,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5741,6 +6663,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5798,6 +6730,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5855,6 +6797,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5912,6 +6864,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5969,6 +6931,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6026,6 +6998,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6083,6 +7065,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6140,6 +7132,16 @@
           <t>D-ADM-03</t>
         </is>
       </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6197,6 +7199,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6254,6 +7266,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6311,6 +7333,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6368,6 +7400,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6425,6 +7467,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6482,6 +7534,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6539,6 +7601,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6596,6 +7668,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6653,6 +7735,16 @@
           <t>D-ADM-02</t>
         </is>
       </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6710,6 +7802,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6767,6 +7869,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6824,6 +7936,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6881,6 +8003,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6938,6 +8070,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6995,6 +8137,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7052,6 +8204,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -7109,6 +8271,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -7166,6 +8338,16 @@
           <t>D-ADM-01</t>
         </is>
       </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -7223,6 +8405,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7280,6 +8472,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -7337,6 +8539,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7394,6 +8606,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7451,6 +8673,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -7508,6 +8740,16 @@
           <t>D-ADM-01</t>
         </is>
       </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -7565,6 +8807,16 @@
           <t>D-ADM-01</t>
         </is>
       </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7622,6 +8874,16 @@
           <t>D-ADM-02</t>
         </is>
       </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>SUT không có Dashboard/revenue API để quan sát hậu điều kiện doanh thu; transition canceled→delivered được phủ riêng bởi TC-024.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7679,6 +8941,16 @@
           <t>D-ADM-03</t>
         </is>
       </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -7736,6 +9008,16 @@
           <t>D-ADM-08</t>
         </is>
       </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -7793,9 +9075,19 @@
           <t>D-ADM-06</t>
         </is>
       </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K129"/>
+  <autoFilter ref="A1:M129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>